<commit_message>
rajout entreprise et rajout mission
</commit_message>
<xml_diff>
--- a/docs/Tableau de compétence BTS SIO SISR Hugo Léonardi.xlsx
+++ b/docs/Tableau de compétence BTS SIO SISR Hugo Léonardi.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
@@ -23,24 +23,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="57" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="68" uniqueCount="41">
   <si>
     <t xml:space="preserve">BTS SERVICES INFORMATIQUES AUX ORGANISATIONS</t>
   </si>
   <si>
-    <t xml:space="preserve">SESSION 2022</t>
+    <t xml:space="preserve">SESSION 2026</t>
   </si>
   <si>
     <t xml:space="preserve">Tableau de synthèse des réalisations professionnelles </t>
   </si>
   <si>
-    <t xml:space="preserve">NOM et prénom : </t>
+    <t xml:space="preserve">NOM et prénom : LEONARDI Hugo</t>
   </si>
   <si>
     <t xml:space="preserve">N° candidat : </t>
   </si>
   <si>
-    <t xml:space="preserve">Centre de formation :</t>
+    <t xml:space="preserve">Centre de formation : Aurlom</t>
   </si>
   <si>
     <t xml:space="preserve">Option :</t>
@@ -52,7 +52,7 @@
     <t xml:space="preserve">▢ SLAM</t>
   </si>
   <si>
-    <t xml:space="preserve">Adresse URL du portfolio : https://bloodsheep000.github.io/portfolio/</t>
+    <t xml:space="preserve">Portfolio : https://hugoleonardi.github.io/portfolio/index.html</t>
   </si>
   <si>
     <t xml:space="preserve">Compétences mises en œuvre
@@ -137,6 +137,12 @@
     <t xml:space="preserve">Veille informatique</t>
   </si>
   <si>
+    <t xml:space="preserve">Infrastructure 3-Tiers Nextcloud sur AWS — Terraform (IaC, EC2, RDS, S3, VPC, IAM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Serveur LLM Self-Hosted — Docker Compose, Caddy, Authelia SSO, Ollama, WireGuard</t>
+  </si>
+  <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de première année</t>
   </si>
   <si>
@@ -147,6 +153,29 @@
   </si>
   <si>
     <t xml:space="preserve">Mise en place d'un serveur Web (Apache, PHP, MySQL - Windows Server 2025)</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Portfolio : </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">https://hugoleonardi.github.io/portfolio/index.html</t>
+    </r>
   </si>
   <si>
     <t xml:space="preserve">Réalisations en milieu professionnel en cours de seconde année</t>
@@ -166,7 +195,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* \-??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -257,6 +286,14 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -266,7 +303,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="21">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -484,6 +521,19 @@
       </top>
       <bottom style="thin">
         <color theme="2" tint="-0.75"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin">
+        <color rgb="FF4A452A"/>
+      </left>
+      <right style="thin"/>
+      <top style="thin">
+        <color rgb="FF4A452A"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF4A452A"/>
       </bottom>
       <diagonal/>
     </border>
@@ -577,7 +627,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -674,23 +724,27 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="17" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -960,7 +1014,7 @@
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:M81"/>
-  <sheetFormatPr defaultColWidth="10.84765625" defaultRowHeight="12.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.84765625" defaultRowHeight="12.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="70.42"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="10.85"/>
@@ -1178,29 +1232,47 @@
       <c r="E13" s="22"/>
       <c r="F13" s="22"/>
       <c r="G13" s="22"/>
-      <c r="H13" s="21" t="s">
+      <c r="H13" s="24" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="14" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19"/>
+      <c r="A14" s="19" t="s">
+        <v>31</v>
+      </c>
       <c r="B14" s="20"/>
-      <c r="C14" s="22"/>
-      <c r="D14" s="22"/>
+      <c r="C14" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D14" s="21"/>
       <c r="E14" s="22"/>
-      <c r="F14" s="22"/>
-      <c r="G14" s="22"/>
-      <c r="H14" s="23"/>
+      <c r="F14" s="22" t="s">
+        <v>26</v>
+      </c>
+      <c r="G14" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="H14" s="24" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="15" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="19"/>
+      <c r="A15" s="19" t="s">
+        <v>32</v>
+      </c>
       <c r="B15" s="20"/>
-      <c r="C15" s="22"/>
-      <c r="D15" s="22"/>
+      <c r="C15" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="D15" s="21"/>
       <c r="E15" s="22"/>
       <c r="F15" s="22"/>
-      <c r="G15" s="22"/>
-      <c r="H15" s="23"/>
+      <c r="G15" s="21" t="s">
+        <v>26</v>
+      </c>
+      <c r="H15" s="24" t="s">
+        <v>26</v>
+      </c>
     </row>
     <row r="16" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="19"/>
@@ -1233,20 +1305,20 @@
       <c r="H18" s="23"/>
     </row>
     <row r="19" s="17" customFormat="true" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
-      <c r="H19" s="24"/>
+      <c r="A19" s="25" t="s">
+        <v>33</v>
+      </c>
+      <c r="B19" s="25"/>
+      <c r="C19" s="25"/>
+      <c r="D19" s="25"/>
+      <c r="E19" s="25"/>
+      <c r="F19" s="25"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
     </row>
     <row r="20" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B20" s="20"/>
       <c r="C20" s="22"/>
@@ -1260,7 +1332,7 @@
     </row>
     <row r="21" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="19" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B21" s="20"/>
       <c r="C21" s="21" t="s">
@@ -1274,7 +1346,7 @@
     </row>
     <row r="22" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="19" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B22" s="20"/>
       <c r="C22" s="21" t="s">
@@ -1291,11 +1363,15 @@
       <c r="H22" s="23"/>
     </row>
     <row r="23" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="19"/>
+      <c r="A23" s="19" t="s">
+        <v>37</v>
+      </c>
       <c r="B23" s="20"/>
       <c r="C23" s="22"/>
       <c r="D23" s="22"/>
-      <c r="E23" s="22"/>
+      <c r="E23" s="21" t="s">
+        <v>26</v>
+      </c>
       <c r="F23" s="22"/>
       <c r="G23" s="22"/>
       <c r="H23" s="23"/>
@@ -1331,20 +1407,20 @@
       <c r="H26" s="23"/>
     </row>
     <row r="27" s="17" customFormat="true" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B27" s="24"/>
-      <c r="C27" s="24"/>
-      <c r="D27" s="24"/>
-      <c r="E27" s="24"/>
-      <c r="F27" s="24"/>
-      <c r="G27" s="24"/>
-      <c r="H27" s="24"/>
+      <c r="A27" s="25" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="25"/>
+      <c r="C27" s="25"/>
+      <c r="D27" s="25"/>
+      <c r="E27" s="25"/>
+      <c r="F27" s="25"/>
+      <c r="G27" s="25"/>
+      <c r="H27" s="25"/>
     </row>
     <row r="28" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="19" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B28" s="20"/>
       <c r="C28" s="22"/>
@@ -1360,7 +1436,7 @@
     </row>
     <row r="29" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="19" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B29" s="20"/>
       <c r="C29" s="21" t="s">
@@ -1417,24 +1493,24 @@
       <c r="H33" s="23"/>
     </row>
     <row r="34" s="17" customFormat="true" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25"/>
-      <c r="B34" s="26"/>
-      <c r="C34" s="27"/>
-      <c r="D34" s="27"/>
-      <c r="E34" s="27"/>
-      <c r="F34" s="27"/>
-      <c r="G34" s="27"/>
-      <c r="H34" s="28"/>
+      <c r="A34" s="26"/>
+      <c r="B34" s="27"/>
+      <c r="C34" s="28"/>
+      <c r="D34" s="28"/>
+      <c r="E34" s="28"/>
+      <c r="F34" s="28"/>
+      <c r="G34" s="28"/>
+      <c r="H34" s="29"/>
     </row>
     <row r="35" s="17" customFormat="true" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="29"/>
-      <c r="B35" s="30"/>
-      <c r="C35" s="31"/>
-      <c r="D35" s="31"/>
-      <c r="E35" s="31"/>
-      <c r="F35" s="31"/>
-      <c r="G35" s="31"/>
-      <c r="H35" s="31"/>
+      <c r="A35" s="30"/>
+      <c r="B35" s="31"/>
+      <c r="C35" s="32"/>
+      <c r="D35" s="32"/>
+      <c r="E35" s="32"/>
+      <c r="F35" s="32"/>
+      <c r="G35" s="32"/>
+      <c r="H35" s="32"/>
     </row>
     <row r="36" s="2" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="37" s="2" customFormat="true" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -1498,7 +1574,7 @@
     <mergeCell ref="A27:H27"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A5" r:id="rId1" display="Adresse URL du portfolio : https://bloodsheep000.github.io/portfolio/"/>
+    <hyperlink ref="A23" r:id="rId1" display="https://hugoleonardi.github.io/portfolio/index.html"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="true" verticalCentered="true"/>
   <pageMargins left="0.196527777777778" right="0.196527777777778" top="0.196527777777778" bottom="0.196527777777778" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>